<commit_message>
Refresh customer intelligence data from updated sample framework Excel across all propositions.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Sample Framework_Customer Database_U.K. Composite Utility Transmission Pole Market.xlsx
+++ b/Sample Framework_Customer Database_U.K. Composite Utility Transmission Pole Market.xlsx
@@ -3,22 +3,34 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87319D97-FC57-4C8E-88A9-B78A5C29FF53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77FD4852-0073-4C75-B573-679955065290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="842" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="842" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="16" r:id="rId1"/>
     <sheet name="Proposition 1 - Basic" sheetId="30" r:id="rId2"/>
     <sheet name="Proposition 2 - Advance" sheetId="29" r:id="rId3"/>
     <sheet name="Proposition 3 - Premium" sheetId="28" r:id="rId4"/>
+    <sheet name="Revised Proposition 3" sheetId="31" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1340" uniqueCount="180">
   <si>
     <t>S.No.</t>
   </si>
@@ -489,13 +501,98 @@
   </si>
   <si>
     <t>https://uk.linkedin.com/in/andrewquail</t>
+  </si>
+  <si>
+    <t>Engineered / composite-alternative pole application for 33 kilovolt distribution overhead-line networks. Public evidence supports UK Power Networks’ engineered pole trial on a 33 kilovolt line.</t>
+  </si>
+  <si>
+    <t>RIIO-2 Electricity Distribution Summary Annual Report: 2023-24</t>
+  </si>
+  <si>
+    <t>Good prospect for composite / engineered pole suppliers, but classify carefully: evidence supports distribution-network engineered pole trial. Priority is medium-high due to network scale, engineering maturity, and potential for asset-standard adoption.</t>
+  </si>
+  <si>
+    <t>https://www.ukpowernetworks.co.uk/</t>
+  </si>
+  <si>
+    <t>Roger Waring</t>
+  </si>
+  <si>
+    <t>roger.waring@ukpowernetworks.co.uk</t>
+  </si>
+  <si>
+    <t>Director of Capital Programme and Procurement</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/roger-waring-5598633/</t>
+  </si>
+  <si>
+    <t>Head of Energy Networks Purchasing</t>
+  </si>
+  <si>
+    <t>neil.harkins@scottishpower.com</t>
+  </si>
+  <si>
+    <t>https://uk.linkedin.com/in/neil-harkins-3b7aba49</t>
+  </si>
+  <si>
+    <t>Mhairi McGilp</t>
+  </si>
+  <si>
+    <t>Category Manager</t>
+  </si>
+  <si>
+    <t>+44 845 270 0700</t>
+  </si>
+  <si>
+    <t>mmcgilp@scottishpower.com</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/mhairi-mcgilp-a5b48346/</t>
+  </si>
+  <si>
+    <t>Paul Leddie</t>
+  </si>
+  <si>
+    <t>p.leddie@sky.com</t>
+  </si>
+  <si>
+    <t>+44 7584 313500</t>
+  </si>
+  <si>
+    <t>Director of Procurement at SSEN Transmission</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/paul-leddie-b27a8b35/</t>
+  </si>
+  <si>
+    <t>NEIL HARKINS 
+(Alternate Person to Contact)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Contact Details </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(Alternate Number can be provided if required)</t>
+    </r>
+  </si>
+  <si>
+    <t>0800 092 9290</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -531,6 +628,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -580,7 +684,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -640,12 +744,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -671,6 +801,10 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -686,6 +820,9 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -693,9 +830,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -707,9 +841,17 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1313,6 +1455,80 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>198438</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>103188</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1492250</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>119063</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Rounded Rectangle 1">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" tooltip="Migrate To Home"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7653CFDB-13E1-4F5E-9EF1-065DB0DA076F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="846138" y="103188"/>
+          <a:ext cx="1903412" cy="777875"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:sysClr val="window" lastClr="FFFFFF"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-IN" sz="2000" b="1" i="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Home</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -1620,90 +1836,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:300" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
     </row>
     <row r="2" spans="1:300" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
     </row>
     <row r="3" spans="1:300" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
     </row>
     <row r="4" spans="1:300" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
     </row>
     <row r="5" spans="1:300" ht="37" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="13" t="s">
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
     </row>
     <row r="6" spans="1:300" ht="130.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="5" t="s">
         <v>27</v>
       </c>
@@ -2642,117 +2858,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:305" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
     </row>
     <row r="2" spans="1:305" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="10"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
     </row>
     <row r="3" spans="1:305" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
     </row>
     <row r="4" spans="1:305" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
+      <c r="A4" s="12"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
     </row>
     <row r="5" spans="1:305" ht="37" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="13" t="s">
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="14" t="s">
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="16"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="19"/>
     </row>
     <row r="6" spans="1:305" ht="130.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11"/>
+      <c r="A6" s="13"/>
       <c r="B6" s="5" t="s">
         <v>27</v>
       </c>
@@ -3922,7 +4138,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83857112-AA1A-47A0-A362-D5D5B4BC2261}">
-  <dimension ref="A1:LD22"/>
+  <dimension ref="A1:LD21"/>
   <sheetFormatPr defaultColWidth="0.1796875" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" customWidth="1"/>
@@ -3947,173 +4163,173 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:316" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
-      <c r="J1" s="10"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="10"/>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
-      <c r="O1" s="10"/>
-      <c r="P1" s="10"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
-      <c r="V1" s="10"/>
-      <c r="W1" s="10"/>
-      <c r="X1" s="10"/>
-      <c r="Y1" s="10"/>
-      <c r="Z1" s="10"/>
-      <c r="AA1" s="10"/>
-      <c r="AB1" s="10"/>
-      <c r="AC1" s="10"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
+      <c r="AA1" s="12"/>
+      <c r="AB1" s="12"/>
+      <c r="AC1" s="12"/>
     </row>
     <row r="2" spans="1:316" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="10"/>
-      <c r="Q2" s="10"/>
-      <c r="R2" s="10"/>
-      <c r="S2" s="10"/>
-      <c r="T2" s="10"/>
-      <c r="U2" s="10"/>
-      <c r="V2" s="10"/>
-      <c r="W2" s="10"/>
-      <c r="X2" s="10"/>
-      <c r="Y2" s="10"/>
-      <c r="Z2" s="10"/>
-      <c r="AA2" s="10"/>
-      <c r="AB2" s="10"/>
-      <c r="AC2" s="10"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="12"/>
+      <c r="AC2" s="12"/>
     </row>
     <row r="3" spans="1:316" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-      <c r="U3" s="10"/>
-      <c r="V3" s="10"/>
-      <c r="W3" s="10"/>
-      <c r="X3" s="10"/>
-      <c r="Y3" s="10"/>
-      <c r="Z3" s="10"/>
-      <c r="AA3" s="10"/>
-      <c r="AB3" s="10"/>
-      <c r="AC3" s="10"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="12"/>
+      <c r="W3" s="12"/>
+      <c r="X3" s="12"/>
+      <c r="Y3" s="12"/>
+      <c r="Z3" s="12"/>
+      <c r="AA3" s="12"/>
+      <c r="AB3" s="12"/>
+      <c r="AC3" s="12"/>
     </row>
     <row r="4" spans="1:316" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="10"/>
-      <c r="T4" s="10"/>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10"/>
-      <c r="W4" s="10"/>
-      <c r="X4" s="10"/>
-      <c r="Y4" s="10"/>
-      <c r="Z4" s="10"/>
-      <c r="AA4" s="10"/>
-      <c r="AB4" s="10"/>
-      <c r="AC4" s="10"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="12"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="12"/>
+      <c r="AB4" s="12"/>
+      <c r="AC4" s="12"/>
     </row>
     <row r="5" spans="1:316" ht="37" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="12"/>
-      <c r="I5" s="13" t="s">
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="14" t="s">
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
-      <c r="S5" s="16"/>
-      <c r="T5" s="18" t="s">
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="U5" s="19"/>
-      <c r="V5" s="19"/>
-      <c r="W5" s="20"/>
-      <c r="X5" s="12" t="s">
+      <c r="U5" s="21"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="Y5" s="12"/>
-      <c r="Z5" s="12"/>
-      <c r="AA5" s="12"/>
-      <c r="AB5" s="17" t="s">
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="14"/>
+      <c r="AA5" s="14"/>
+      <c r="AB5" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="AC5" s="17"/>
+      <c r="AC5" s="16"/>
     </row>
     <row r="6" spans="1:316" ht="130.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="11"/>
+      <c r="B6" s="13"/>
       <c r="C6" s="5" t="s">
         <v>27</v>
       </c>
@@ -4198,7 +4414,7 @@
       <c r="DQ6" s="2"/>
     </row>
     <row r="7" spans="1:316" s="2" customFormat="1" ht="174.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="9" t="s">
         <v>101</v>
       </c>
       <c r="B7" s="3">
@@ -4547,7 +4763,7 @@
       <c r="LD7"/>
     </row>
     <row r="8" spans="1:316" s="2" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="9" t="s">
         <v>130</v>
       </c>
       <c r="B8" s="3">
@@ -4636,7 +4852,7 @@
       </c>
     </row>
     <row r="9" spans="1:316" s="2" customFormat="1" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="9" t="s">
         <v>100</v>
       </c>
       <c r="B9" s="3">
@@ -4725,7 +4941,7 @@
       </c>
     </row>
     <row r="10" spans="1:316" s="2" customFormat="1" ht="145" x14ac:dyDescent="0.35">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="10" t="s">
         <v>98</v>
       </c>
       <c r="B10" s="3">
@@ -6019,7 +6235,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:29" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B1:AC4"/>
@@ -6041,4 +6256,1859 @@
   <pageSetup orientation="portrait" r:id="rId5"/>
   <drawing r:id="rId6"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0E1D811-130D-4D5E-81FF-8889CC0A21B2}">
+  <dimension ref="A1:LD24"/>
+  <sheetFormatPr defaultColWidth="0.1796875" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.26953125" customWidth="1"/>
+    <col min="2" max="2" width="8.7265625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.26953125" customWidth="1"/>
+    <col min="5" max="5" width="28.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="14" width="16.1796875" customWidth="1"/>
+    <col min="15" max="15" width="27.54296875" customWidth="1"/>
+    <col min="16" max="16" width="25.453125" customWidth="1"/>
+    <col min="17" max="19" width="20.1796875" customWidth="1"/>
+    <col min="20" max="20" width="24.54296875" customWidth="1"/>
+    <col min="21" max="21" width="16.1796875" customWidth="1"/>
+    <col min="22" max="23" width="19.26953125" customWidth="1"/>
+    <col min="24" max="24" width="24.453125" customWidth="1"/>
+    <col min="25" max="26" width="25.7265625" customWidth="1"/>
+    <col min="27" max="27" width="21.1796875" customWidth="1"/>
+    <col min="28" max="28" width="18.26953125" customWidth="1"/>
+    <col min="29" max="29" width="16.1796875" customWidth="1"/>
+    <col min="30" max="30" width="0.1796875" customWidth="1"/>
+    <col min="34" max="34" width="0.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:316" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
+      <c r="AA1" s="12"/>
+      <c r="AB1" s="12"/>
+      <c r="AC1" s="12"/>
+    </row>
+    <row r="2" spans="1:316" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="12"/>
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="12"/>
+      <c r="AB2" s="12"/>
+      <c r="AC2" s="12"/>
+    </row>
+    <row r="3" spans="1:316" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12"/>
+      <c r="T3" s="12"/>
+      <c r="U3" s="12"/>
+      <c r="V3" s="12"/>
+      <c r="W3" s="12"/>
+      <c r="X3" s="12"/>
+      <c r="Y3" s="12"/>
+      <c r="Z3" s="12"/>
+      <c r="AA3" s="12"/>
+      <c r="AB3" s="12"/>
+      <c r="AC3" s="12"/>
+    </row>
+    <row r="4" spans="1:316" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12"/>
+      <c r="T4" s="12"/>
+      <c r="U4" s="12"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="12"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="12"/>
+      <c r="AB4" s="12"/>
+      <c r="AC4" s="12"/>
+    </row>
+    <row r="5" spans="1:316" ht="37" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="U5" s="21"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="Y5" s="14"/>
+      <c r="Z5" s="14"/>
+      <c r="AA5" s="14"/>
+      <c r="AB5" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="AC5" s="16"/>
+    </row>
+    <row r="6" spans="1:316" ht="130.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="13"/>
+      <c r="C6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="R6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="S6" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="T6" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="U6" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="V6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="W6" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB6" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="DQ6" s="2"/>
+    </row>
+    <row r="7" spans="1:316" s="2" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="3">
+        <v>2</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="K7" s="24" t="s">
+        <v>161</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="M7" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="N7" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="S7" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="U7" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="V7" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="W7" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="X7" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="Y7" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="Z7" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="AA7" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="AB7" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="AC7" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="8" spans="1:316" s="2" customFormat="1" ht="130.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="3">
+        <v>3</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="G8" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="M8" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="N8" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="O8" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="P8" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q8" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="R8" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="S8" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="T8" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="U8" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="V8" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="W8" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="X8" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y8" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z8" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="AA8" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="AB8" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="AC8" s="25" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:316" s="2" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="9"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="K9" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="M9" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="N9" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="O9" s="26"/>
+      <c r="P9" s="26"/>
+      <c r="Q9" s="26"/>
+      <c r="R9" s="26"/>
+      <c r="S9" s="26"/>
+      <c r="T9" s="26"/>
+      <c r="U9" s="26"/>
+      <c r="V9" s="26"/>
+      <c r="W9" s="26"/>
+      <c r="X9" s="26"/>
+      <c r="Y9" s="26"/>
+      <c r="Z9" s="26"/>
+      <c r="AA9" s="26"/>
+      <c r="AB9" s="26"/>
+      <c r="AC9" s="26"/>
+    </row>
+    <row r="10" spans="1:316" s="2" customFormat="1" ht="145" x14ac:dyDescent="0.35">
+      <c r="A10" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="3">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="K10" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="M10" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="N10" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="P10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q10" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="R10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="S10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="T10" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="U10" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="V10" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="W10" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="X10" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="Y10" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AA10" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="AB10" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="AC10" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="BE10"/>
+      <c r="BF10"/>
+      <c r="BG10"/>
+      <c r="BH10"/>
+      <c r="BI10"/>
+      <c r="BJ10"/>
+      <c r="BK10"/>
+      <c r="BL10"/>
+      <c r="BM10"/>
+      <c r="BN10"/>
+      <c r="BO10"/>
+      <c r="BP10"/>
+      <c r="BQ10"/>
+      <c r="BR10"/>
+      <c r="BS10"/>
+      <c r="BT10"/>
+      <c r="BU10"/>
+      <c r="BV10"/>
+      <c r="BW10"/>
+      <c r="BX10"/>
+      <c r="BY10"/>
+      <c r="BZ10"/>
+      <c r="CA10"/>
+      <c r="CB10"/>
+      <c r="CC10"/>
+      <c r="CD10"/>
+      <c r="CE10"/>
+      <c r="CF10"/>
+      <c r="CG10"/>
+      <c r="CH10"/>
+      <c r="CI10"/>
+      <c r="CJ10"/>
+      <c r="CK10"/>
+      <c r="CL10"/>
+      <c r="CM10"/>
+      <c r="CN10"/>
+      <c r="CO10"/>
+      <c r="CP10"/>
+      <c r="CQ10"/>
+      <c r="CR10"/>
+      <c r="CS10"/>
+      <c r="CT10"/>
+      <c r="CU10"/>
+      <c r="CV10"/>
+      <c r="CW10"/>
+      <c r="CX10"/>
+      <c r="CY10"/>
+      <c r="CZ10"/>
+      <c r="DA10"/>
+      <c r="DB10"/>
+      <c r="DC10"/>
+      <c r="DD10"/>
+      <c r="DE10"/>
+      <c r="DF10"/>
+      <c r="DG10"/>
+      <c r="DH10"/>
+      <c r="DI10"/>
+      <c r="DJ10"/>
+      <c r="DK10"/>
+      <c r="DL10"/>
+      <c r="DM10"/>
+      <c r="DN10"/>
+      <c r="DO10"/>
+      <c r="DP10"/>
+      <c r="DQ10"/>
+      <c r="DR10"/>
+      <c r="DS10"/>
+      <c r="DT10"/>
+      <c r="DU10"/>
+      <c r="DV10"/>
+      <c r="DW10"/>
+      <c r="DX10"/>
+      <c r="DY10"/>
+      <c r="DZ10"/>
+      <c r="EA10"/>
+      <c r="EB10"/>
+      <c r="EC10"/>
+      <c r="ED10"/>
+      <c r="EE10"/>
+      <c r="EF10"/>
+      <c r="EG10"/>
+      <c r="EH10"/>
+      <c r="EI10"/>
+      <c r="EJ10"/>
+      <c r="EK10"/>
+      <c r="EL10"/>
+      <c r="EM10"/>
+      <c r="EN10"/>
+      <c r="EO10"/>
+      <c r="EP10"/>
+      <c r="EQ10"/>
+      <c r="ER10"/>
+      <c r="ES10"/>
+      <c r="ET10"/>
+      <c r="EU10"/>
+      <c r="EV10"/>
+      <c r="EW10"/>
+      <c r="EX10"/>
+      <c r="EY10"/>
+      <c r="EZ10"/>
+      <c r="FA10"/>
+      <c r="FB10"/>
+      <c r="FC10"/>
+      <c r="FD10"/>
+      <c r="FE10"/>
+      <c r="FF10"/>
+      <c r="FG10"/>
+      <c r="FH10"/>
+      <c r="FI10"/>
+      <c r="FJ10"/>
+      <c r="FK10"/>
+      <c r="FL10"/>
+      <c r="FM10"/>
+      <c r="FN10"/>
+      <c r="FO10"/>
+      <c r="FP10"/>
+      <c r="FQ10"/>
+      <c r="FR10"/>
+      <c r="FS10"/>
+      <c r="FT10"/>
+      <c r="FU10"/>
+      <c r="FV10"/>
+      <c r="FW10"/>
+      <c r="FX10"/>
+      <c r="FY10"/>
+      <c r="FZ10"/>
+      <c r="GA10"/>
+      <c r="GB10"/>
+      <c r="GC10"/>
+      <c r="GD10"/>
+      <c r="GE10"/>
+      <c r="GF10"/>
+      <c r="GG10"/>
+      <c r="GH10"/>
+      <c r="GI10"/>
+      <c r="GJ10"/>
+      <c r="GK10"/>
+      <c r="GL10"/>
+      <c r="GM10"/>
+      <c r="GN10"/>
+      <c r="GO10"/>
+      <c r="GP10"/>
+      <c r="GQ10"/>
+      <c r="GR10"/>
+      <c r="GS10"/>
+      <c r="GT10"/>
+      <c r="GU10"/>
+      <c r="GV10"/>
+      <c r="GW10"/>
+      <c r="GX10"/>
+      <c r="GY10"/>
+      <c r="GZ10"/>
+      <c r="HA10"/>
+      <c r="HB10"/>
+      <c r="HC10"/>
+      <c r="HD10"/>
+      <c r="HE10"/>
+      <c r="HF10"/>
+      <c r="HG10"/>
+      <c r="HH10"/>
+      <c r="HI10"/>
+      <c r="HJ10"/>
+      <c r="HK10"/>
+      <c r="HL10"/>
+      <c r="HM10"/>
+      <c r="HN10"/>
+      <c r="HO10"/>
+      <c r="HP10"/>
+      <c r="HQ10"/>
+      <c r="HR10"/>
+      <c r="HS10"/>
+      <c r="HT10"/>
+      <c r="HU10"/>
+      <c r="HV10"/>
+      <c r="HW10"/>
+      <c r="HX10"/>
+      <c r="HY10"/>
+      <c r="HZ10"/>
+      <c r="IA10"/>
+      <c r="IB10"/>
+      <c r="IC10"/>
+      <c r="ID10"/>
+      <c r="IE10"/>
+      <c r="IF10"/>
+      <c r="IG10"/>
+      <c r="IH10"/>
+      <c r="II10"/>
+      <c r="IJ10"/>
+      <c r="IK10"/>
+      <c r="IL10"/>
+      <c r="IM10"/>
+      <c r="IN10"/>
+      <c r="IO10"/>
+      <c r="IP10"/>
+      <c r="IQ10"/>
+      <c r="IR10"/>
+      <c r="IS10"/>
+      <c r="IT10"/>
+      <c r="IU10"/>
+      <c r="IV10"/>
+      <c r="IW10"/>
+      <c r="IX10"/>
+      <c r="IY10"/>
+      <c r="IZ10"/>
+      <c r="JA10"/>
+      <c r="JB10"/>
+      <c r="JC10"/>
+      <c r="JD10"/>
+      <c r="JE10"/>
+      <c r="JF10"/>
+      <c r="JG10"/>
+      <c r="JH10"/>
+      <c r="JI10"/>
+      <c r="JJ10"/>
+      <c r="JK10"/>
+      <c r="JL10"/>
+      <c r="JM10"/>
+      <c r="JN10"/>
+      <c r="JO10"/>
+      <c r="JP10"/>
+      <c r="JQ10"/>
+      <c r="JR10"/>
+      <c r="JS10"/>
+      <c r="JT10"/>
+      <c r="JU10"/>
+      <c r="JV10"/>
+      <c r="JW10"/>
+      <c r="JX10"/>
+      <c r="JY10"/>
+      <c r="JZ10"/>
+      <c r="KA10"/>
+      <c r="KB10"/>
+      <c r="KC10"/>
+      <c r="KD10"/>
+      <c r="KE10"/>
+      <c r="KF10"/>
+      <c r="KG10"/>
+      <c r="KH10"/>
+      <c r="KI10"/>
+      <c r="KJ10"/>
+      <c r="KK10"/>
+      <c r="KL10"/>
+      <c r="KM10"/>
+      <c r="KN10"/>
+      <c r="KO10"/>
+      <c r="KP10"/>
+      <c r="KQ10"/>
+      <c r="KR10"/>
+      <c r="KS10"/>
+      <c r="KT10"/>
+      <c r="KU10"/>
+      <c r="KV10"/>
+      <c r="KW10"/>
+      <c r="KX10"/>
+      <c r="KY10"/>
+      <c r="KZ10"/>
+      <c r="LA10"/>
+      <c r="LB10"/>
+      <c r="LC10"/>
+      <c r="LD10"/>
+    </row>
+    <row r="11" spans="1:316" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="3">
+        <v>5</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB11" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC11" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:316" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="3">
+        <v>6</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC12" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:316" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="3">
+        <v>7</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB13" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC13" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:316" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="3">
+        <v>8</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC14" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:316" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="3">
+        <v>9</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB15" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC15" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:316" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="3">
+        <v>10</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB16" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC16" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:29" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="3">
+        <v>11</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC17" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:29" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="3">
+        <v>12</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB18" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC18" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:29" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="3">
+        <v>13</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB19" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC19" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:29" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="3">
+        <v>14</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB20" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC20" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:29" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="3">
+        <v>15</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="N21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="O21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="P21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="R21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="S21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="T21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="U21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="V21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="W21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="X21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB21" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="AC21" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:29" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="24" spans="2:29" ht="0" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
+  </sheetData>
+  <mergeCells count="29">
+    <mergeCell ref="AA8:AA9"/>
+    <mergeCell ref="AB8:AB9"/>
+    <mergeCell ref="AC8:AC9"/>
+    <mergeCell ref="U8:U9"/>
+    <mergeCell ref="V8:V9"/>
+    <mergeCell ref="W8:W9"/>
+    <mergeCell ref="X8:X9"/>
+    <mergeCell ref="Y8:Y9"/>
+    <mergeCell ref="Z8:Z9"/>
+    <mergeCell ref="O8:O9"/>
+    <mergeCell ref="P8:P9"/>
+    <mergeCell ref="Q8:Q9"/>
+    <mergeCell ref="R8:R9"/>
+    <mergeCell ref="S8:S9"/>
+    <mergeCell ref="T8:T9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="B1:AC4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="I5:N5"/>
+    <mergeCell ref="O5:S5"/>
+    <mergeCell ref="T5:W5"/>
+    <mergeCell ref="X5:AA5"/>
+    <mergeCell ref="AB5:AC5"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A10" r:id="rId1" display="https://www.ssen-transmission.co.uk/news/news--views/2018/2/flying-into-pole-position/" xr:uid="{89338927-62E9-491D-9AFF-6EDB5DD96C9D}"/>
+    <hyperlink ref="A8" r:id="rId2" display="https://smarter.energynetworks.org/projects/nia_spen0019/" xr:uid="{39E70573-7C1F-420D-9184-94FAF59D0FD9}"/>
+    <hyperlink ref="A7" r:id="rId3" display="https://smarter.energynetworks.org/projects/nia_ukpn0039/" xr:uid="{D561FA08-F9D3-44E4-80F1-6CB32E6C5941}"/>
+    <hyperlink ref="A5" r:id="rId4" display="https://www.ofgem.gov.uk/sites/default/files/2025-04/RIIO-2 Electricity Distribution Annual Report 2023 to 2024.pdf" xr:uid="{3A415AF2-5234-4138-978E-A4F9B53FEEDE}"/>
+    <hyperlink ref="N8" r:id="rId5" xr:uid="{A5D46240-486F-4961-A929-5D5B24331C10}"/>
+    <hyperlink ref="N10" r:id="rId6" xr:uid="{00AECD38-5FC4-43D2-92CC-1D10F1CD59E3}"/>
+    <hyperlink ref="N7" r:id="rId7" xr:uid="{9A9C54A3-4A83-4401-B0C5-534B312335C2}"/>
+    <hyperlink ref="K7" r:id="rId8" display="mailto:roger.waring@ukpowernetworks.co.uk" xr:uid="{12E92FB4-746E-4D00-806A-75CAD295C918}"/>
+    <hyperlink ref="M7" r:id="rId9" xr:uid="{806DF0AB-DE0D-4216-BE5A-31F314071FB0}"/>
+    <hyperlink ref="K9" r:id="rId10" xr:uid="{3B7C4373-E711-4F9F-A4C1-09944F6FCEF8}"/>
+    <hyperlink ref="M9" r:id="rId11" xr:uid="{E59CADBA-91A0-4B04-99E1-3B0A847F98DE}"/>
+    <hyperlink ref="N9" r:id="rId12" xr:uid="{4FCF010E-55A1-4EAE-97A8-D18F0F4AE26F}"/>
+    <hyperlink ref="K8" r:id="rId13" xr:uid="{97D210EF-B880-4FE2-BFAC-275AA37D57AA}"/>
+    <hyperlink ref="M8" r:id="rId14" xr:uid="{2AC1DA5C-749B-4204-96A3-09E3173649FB}"/>
+    <hyperlink ref="K10" r:id="rId15" xr:uid="{9EB5C8CE-2925-494C-83CF-961A9D4CBA55}"/>
+    <hyperlink ref="M10" r:id="rId16" xr:uid="{6A392515-9321-4D67-91A4-B214ADBE13C8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId17"/>
+  <drawing r:id="rId18"/>
+</worksheet>
 </file>
</xml_diff>